<commit_message>
Credit DOE/NREL/ALLIANCE as the Databank notice requires
The Battery Failure Databank notice asks every publication that results
from the data to credit DOE/NREL/ALLIANCE. The credit now appears as a
line at the end of the note (PDF re-rendered, still one page) and in the
README's Databank source entry. The results workbook, whose sheet
Databank rows used copies Databank rows, now carries the notice in full
on a sheet of its own, with the same credit on its Read me sheet.
CITATION.cff gains the author's ORCID.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JRQdFboVN1WcGEdwURaRN7
</commit_message>
<xml_diff>
--- a/results/m50_two_cell_results.xlsx
+++ b/results/m50_two_cell_results.xlsx
@@ -14,8 +14,9 @@
     <sheet name="Resolved one strip" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Scorecard" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Databank rows used" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Verification" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Exploratory" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Databank notice" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Verification" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Exploratory" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="187">
   <si>
     <t xml:space="preserve">Where and when a neighbour cell first reaches thermal-runaway onset temperatures: resolved against lumped, a pre-registered two-cell LG M50 pilot. Repository github.com/siddharth161204-wq/m50-two-cell-pilot</t>
   </si>
@@ -53,6 +54,12 @@
     <t xml:space="preserve">Columns in blue on 'Resolved two strips' are formulas: time saved and ratio at 183.5 C where both models cross.</t>
   </si>
   <si>
+    <t xml:space="preserve">The sheet Databank rows used copies rows of the Battery Failure Databank; the Databank's notice is reproduced in full on the sheet Databank notice and must accompany every copy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Battery Failure Databank is provided by the U.S. Department of Energy's National Renewable Energy Laboratory, operated by Alliance for Sustainable Energy, LLC (DOE/NREL/ALLIANCE); its notice accompanies the rows used, in inputs/databank/.</t>
+  </si>
+  <si>
     <t xml:space="preserve">E_body (J)</t>
   </si>
   <si>
@@ -387,6 +394,18 @@
   </si>
   <si>
     <t xml:space="preserve">SPR2021_ESTA_8B100-01_SOC_RUN198</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The rows in databank_m50_rows.csv are copied unchanged from the Battery Failure Databank (sheet "Battery Failure Databank", all rows whose Cell-Description contains "M50"). The Databank's own notice, reproduced in full as it requires:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The National Renewable Energy Laboratory (NREL) is operated for the U.S. Department of Energy (DOE) by Alliance for Sustainable Energy, LLC ("Alliance").</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access to or use of any data or software made available on this server ("Data") shall impose the following obligations on the user, and use of the Data constitutes user's agreement to these terms. The user is granted the right, without any fee or cost, to use or copy the Data, provided that this entire notice appears in all copies of the Data. Further, the user agrees to credit DOE/NREL/ALLIANCE in any publication that results from the use of the Data. The names DOE/NREL/ALLIANCE, however, may not be used in any advertising or publicity to endorse or promote any products or commercial entities unless specific written permission is obtained from DOE/NREL/ ALLIANCE. The user also understands that DOE/NREL/ALLIANCE are not obligated to provide the user with any support, consulting, training or assistance of any kind with regard to the use of the Data or to provide the user with any updates, revisions or new versions thereof. DOE, NREL, and ALLIANCE do not guarantee or endorse any results generated by use of the Data, and user is entirely responsible for the results and any reliance on the results or the Data in general.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USER AGREES TO INDEMNIFY DOE/NREL/ALLIANCE AND ITS SUBSIDIARIES, AFFILIATES, OFFICERS, AGENTS, AND EMPLOYEES AGAINST ANY CLAIM OR DEMAND, INCLUDING REASONABLE ATTORNEYS' FEES, RELATED TO USER'S USE OF THE DATA. THE DATA ARE PROVIDED BY DOE/NREL/ALLIANCE "AS IS," AND ANY EXPRESS OR IMPLIED WARRANTIES, INCLUDING BUT NOT LIMITED TO THE IMPLIED WARRANTIES OF MERCHANTABILITY AND FITNESS FOR A PARTICULAR PURPOSE ARE DISCLAIMED. DOE/NREL/ALLIANCE ASSUME NO LEGAL LIABILITY OR RESPONSIBILITY FOR THE ACCURACY, COMPLETENESS, OR USEFULNESS OF THE DATA, OR REPRESENT THAT ITS USE WOULD NOT INFRINGE PRIVATELY OWNED RIGHTS. IN NO EVENT SHALL DOE/NREL/ALLIANCE BE LIABLE FOR ANY SPECIAL, INDIRECT OR CONSEQUENTIAL DAMAGES OR ANY DAMAGES WHATSOEVER, INCLUDING BUT NOT LIMITED TO CLAIMS ASSOCIATED WITH THE LOSS OF DATA OR PROFITS, THAT MAY RESULT FROM AN ACTION IN CONTRACT, NEGLIGENCE OR OTHER TORTIOUS CLAIM THAT ARISES OUT OF OR IN CONNECTION WITH THE ACCESS, USE OR PERFORMANCE OF THE DATA.</t>
   </si>
   <si>
     <t xml:space="preserve">Check</t>
@@ -674,7 +693,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -693,6 +712,10 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -955,7 +978,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="150"/>
@@ -999,6 +1022,16 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1030,43 +1063,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2361,133 +2394,133 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AB1" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="AD1" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AE1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="AF1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AG1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="AH1" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="AI1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="AJ1" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="AK1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="AL1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="AM1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="AN1" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="AO1" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="AP1" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AQ1" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2516,10 +2549,10 @@
         <v>578.3</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -2589,10 +2622,10 @@
         <v>565.5</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -2662,10 +2695,10 @@
         <v>475.7</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -2735,10 +2768,10 @@
         <v>310.3</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -2808,10 +2841,10 @@
         <v>134.8</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -2881,10 +2914,10 @@
         <v>29.3</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -2954,10 +2987,10 @@
         <v>15.9</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
@@ -3027,10 +3060,10 @@
         <v>588.5</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
@@ -3100,10 +3133,10 @@
         <v>575.8</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
@@ -3173,10 +3206,10 @@
         <v>486</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -3246,10 +3279,10 @@
         <v>320.4</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -3319,10 +3352,10 @@
         <v>144.9</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -3392,10 +3425,10 @@
         <v>41.5</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -3465,10 +3498,10 @@
         <v>30.6</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -3538,10 +3571,10 @@
         <v>476</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
@@ -3611,10 +3644,10 @@
         <v>483.1</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
@@ -3684,10 +3717,10 @@
         <v>407.3</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -3757,10 +3790,10 @@
         <v>258.8</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
@@ -3830,10 +3863,10 @@
         <v>59.2</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
@@ -3903,10 +3936,10 @@
         <v>26.6</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2" t="n">
@@ -3914,7 +3947,7 @@
       </c>
       <c r="M21" s="2"/>
       <c r="N21" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O21" s="2" t="n">
         <v>132.97</v>
@@ -3982,10 +4015,10 @@
         <v>15.4</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K22" s="2"/>
       <c r="L22" s="2" t="n">
@@ -3993,7 +4026,7 @@
       </c>
       <c r="M22" s="2"/>
       <c r="N22" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O22" s="2" t="n">
         <v>141.03</v>
@@ -4004,7 +4037,7 @@
       </c>
       <c r="R22" s="2"/>
       <c r="S22" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T22" s="2" t="n">
         <v>154.34</v>
@@ -4015,7 +4048,7 @@
       </c>
       <c r="W22" s="2"/>
       <c r="X22" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Y22" s="2" t="n">
         <v>168.12</v>
@@ -4073,10 +4106,10 @@
         <v>486.6</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -4146,10 +4179,10 @@
         <v>493.7</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
@@ -4219,10 +4252,10 @@
         <v>417.6</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -4292,10 +4325,10 @@
         <v>269</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -4365,10 +4398,10 @@
         <v>70.4</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
@@ -4438,10 +4471,10 @@
         <v>39</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K28" s="2"/>
       <c r="L28" s="2" t="n">
@@ -4449,7 +4482,7 @@
       </c>
       <c r="M28" s="2"/>
       <c r="N28" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O28" s="2" t="n">
         <v>130.2</v>
@@ -4517,10 +4550,10 @@
         <v>30.3</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2" t="n">
@@ -4528,7 +4561,7 @@
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O29" s="2" t="n">
         <v>135.65</v>
@@ -4539,7 +4572,7 @@
       </c>
       <c r="R29" s="2"/>
       <c r="S29" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T29" s="2" t="n">
         <v>148.23</v>
@@ -4550,7 +4583,7 @@
       </c>
       <c r="W29" s="2"/>
       <c r="X29" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Y29" s="2" t="n">
         <v>160.64</v>
@@ -4608,10 +4641,10 @@
         <v>390</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
@@ -4681,10 +4714,10 @@
         <v>415.4</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
@@ -4754,10 +4787,10 @@
         <v>350.7</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
@@ -4827,10 +4860,10 @@
         <v>215</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
@@ -4900,10 +4933,10 @@
         <v>39.7</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K34" s="2"/>
       <c r="L34" s="2" t="n">
@@ -4911,7 +4944,7 @@
       </c>
       <c r="M34" s="2"/>
       <c r="N34" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O34" s="2" t="n">
         <v>127.71</v>
@@ -4979,10 +5012,10 @@
         <v>23.9</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K35" s="2"/>
       <c r="L35" s="2" t="n">
@@ -4990,7 +5023,7 @@
       </c>
       <c r="M35" s="2"/>
       <c r="N35" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O35" s="2" t="n">
         <v>139.51</v>
@@ -5001,7 +5034,7 @@
       </c>
       <c r="R35" s="2"/>
       <c r="S35" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T35" s="2" t="n">
         <v>153.53</v>
@@ -5012,7 +5045,7 @@
       </c>
       <c r="W35" s="2"/>
       <c r="X35" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Y35" s="2" t="n">
         <v>167.25</v>
@@ -5070,10 +5103,10 @@
         <v>14.8</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>57.46</v>
@@ -5083,7 +5116,7 @@
       </c>
       <c r="M36" s="2"/>
       <c r="N36" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O36" s="2" t="n">
         <v>143.82</v>
@@ -5096,7 +5129,7 @@
       </c>
       <c r="R36" s="2"/>
       <c r="S36" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T36" s="2" t="n">
         <v>154.43</v>
@@ -5109,7 +5142,7 @@
       </c>
       <c r="W36" s="2"/>
       <c r="X36" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Y36" s="2" t="n">
         <v>170.03</v>
@@ -5120,7 +5153,7 @@
       </c>
       <c r="AB36" s="2"/>
       <c r="AC36" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="AD36" s="2" t="n">
         <v>226.06</v>
@@ -5131,7 +5164,7 @@
       </c>
       <c r="AG36" s="2"/>
       <c r="AH36" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="AI36" s="2" t="n">
         <v>245.47</v>
@@ -5142,7 +5175,7 @@
       </c>
       <c r="AL36" s="2"/>
       <c r="AM36" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="AN36" s="2" t="n">
         <v>268.13</v>
@@ -5185,10 +5218,10 @@
         <v>400.8</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
@@ -5258,10 +5291,10 @@
         <v>426.1</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
@@ -5331,10 +5364,10 @@
         <v>361.2</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
@@ -5404,10 +5437,10 @@
         <v>225.2</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
@@ -5477,10 +5510,10 @@
         <v>51.2</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K41" s="2"/>
       <c r="L41" s="2" t="n">
@@ -5488,7 +5521,7 @@
       </c>
       <c r="M41" s="2"/>
       <c r="N41" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O41" s="2" t="n">
         <v>126.85</v>
@@ -5556,10 +5589,10 @@
         <v>36.5</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K42" s="2"/>
       <c r="L42" s="2" t="n">
@@ -5567,7 +5600,7 @@
       </c>
       <c r="M42" s="2"/>
       <c r="N42" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O42" s="2" t="n">
         <v>136.43</v>
@@ -5578,7 +5611,7 @@
       </c>
       <c r="R42" s="2"/>
       <c r="S42" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T42" s="2" t="n">
         <v>149.72</v>
@@ -5589,7 +5622,7 @@
       </c>
       <c r="W42" s="2"/>
       <c r="X42" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Y42" s="2" t="n">
         <v>161.55</v>
@@ -5647,10 +5680,10 @@
         <v>30</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>67.3</v>
@@ -5660,7 +5693,7 @@
       </c>
       <c r="M43" s="2"/>
       <c r="N43" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O43" s="2" t="n">
         <v>138.31</v>
@@ -5673,7 +5706,7 @@
       </c>
       <c r="R43" s="2"/>
       <c r="S43" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T43" s="2" t="n">
         <v>151.94</v>
@@ -5686,7 +5719,7 @@
       </c>
       <c r="W43" s="2"/>
       <c r="X43" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Y43" s="2" t="n">
         <v>165.4</v>
@@ -5697,7 +5730,7 @@
       </c>
       <c r="AB43" s="2"/>
       <c r="AC43" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="AD43" s="2" t="n">
         <v>216.69</v>
@@ -5708,7 +5741,7 @@
       </c>
       <c r="AG43" s="2"/>
       <c r="AH43" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="AI43" s="2" t="n">
         <v>236.14</v>
@@ -5719,7 +5752,7 @@
       </c>
       <c r="AL43" s="2"/>
       <c r="AM43" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="AN43" s="2" t="n">
         <v>256.52</v>
@@ -5795,124 +5828,124 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="AB1" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="AD1" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="AE1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="AF1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AG1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="AH1" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="AI1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="AJ1" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="AK1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="AL1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="AM1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="AN1" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5941,10 +5974,10 @@
         <v>460.7</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -6003,10 +6036,10 @@
         <v>425.4</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -6065,10 +6098,10 @@
         <v>362.1</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -6127,10 +6160,10 @@
         <v>222.1</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -6189,10 +6222,10 @@
         <v>120.7</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -6251,10 +6284,10 @@
         <v>68.3</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -6313,10 +6346,10 @@
         <v>37.1</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2" t="n">
@@ -6324,7 +6357,7 @@
       </c>
       <c r="M8" s="2"/>
       <c r="N8" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O8" s="2" t="n">
         <v>130.81</v>
@@ -6335,7 +6368,7 @@
       </c>
       <c r="R8" s="2"/>
       <c r="S8" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T8" s="2" t="n">
         <v>142.28</v>
@@ -6346,7 +6379,7 @@
       </c>
       <c r="W8" s="2"/>
       <c r="X8" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Y8" s="2" t="n">
         <v>152.42</v>
@@ -6394,86 +6427,86 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -6510,48 +6543,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>4.171</v>
@@ -6581,15 +6614,15 @@
         <v>45.9545</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>4.162</v>
@@ -6619,15 +6652,15 @@
         <v>53.8874</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>4.175</v>
@@ -6657,15 +6690,15 @@
         <v>44.7723</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>4.16</v>
@@ -6695,15 +6728,15 @@
         <v>38.9573</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>4.174</v>
@@ -6733,15 +6766,15 @@
         <v>34.5351</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>4.171</v>
@@ -6771,15 +6804,15 @@
         <v>30.4219</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>4.172</v>
@@ -6809,15 +6842,15 @@
         <v>45.6915</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>4.164</v>
@@ -6847,15 +6880,15 @@
         <v>40.8514</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>4.174</v>
@@ -6885,15 +6918,15 @@
         <v>33.5084</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>4.17</v>
@@ -6923,15 +6956,15 @@
         <v>33.9934</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>4.174</v>
@@ -6961,15 +6994,15 @@
         <v>35.9844</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>4.189</v>
@@ -6999,15 +7032,15 @@
         <v>41.7189</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>4.1797</v>
@@ -7037,15 +7070,15 @@
         <v>39.87</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>4.1768</v>
@@ -7075,15 +7108,15 @@
         <v>40.4</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>4.1757</v>
@@ -7113,15 +7146,15 @@
         <v>41.64</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>4.176</v>
@@ -7151,15 +7184,15 @@
         <v>47.08</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>4.1727</v>
@@ -7189,7 +7222,7 @@
         <v>48.85</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -7208,243 +7241,30 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="160"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>121</v>
+    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>0.975717875127543</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A2" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>2.32108658728963E-011</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>-0.00064855625061</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>125</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>0.000819881202914985</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>0.206181815170737</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>-0.0217247255258144</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>0.00503790786554426</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>0.062616266371947</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>0.00548299125347285</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>0.0200216726846616</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>1.48897783640496</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>-0.305821865303415</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>0.00327365881429564</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>0.0398145369898657</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>0.00551631911679351</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>0.0847956586240528</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>1.41088468164253</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>-0.307861475483378</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>85.700699276118</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>82.9629522175588</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>96.718297592367</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>1.2E-011</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>0.308102760535576</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="B29" s="2" t="n">
-        <v>0.169868364338555</v>
       </c>
     </row>
   </sheetData>
@@ -7459,6 +7279,261 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B29"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>0.975717875127543</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>2.32108658728963E-011</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>-0.00064855625061</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0.000819881202914985</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>0.206181815170737</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>-0.0217247255258144</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>0.00503790786554426</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0.062616266371947</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0.00548299125347285</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>0.0200216726846616</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>1.48897783640496</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>-0.305821865303415</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>0.00327365881429564</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>0.0398145369898657</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>0.00551631911679351</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>0.0847956586240528</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>1.41088468164253</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>-0.307861475483378</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>85.700699276118</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>82.9629522175588</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>96.718297592367</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>1.2E-011</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>0.308102760535576</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>0.169868364338555</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -7484,57 +7559,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>33222.9</v>
@@ -7579,12 +7654,12 @@
         <v>506.551464304854</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>33222.9</v>
@@ -7629,12 +7704,12 @@
         <v>540.007305810652</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>21495.3</v>
@@ -7664,7 +7739,7 @@
         <v>134.023204376743</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>152.8</v>
@@ -7679,12 +7754,12 @@
         <v>340.182758683711</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>33222.9</v>
@@ -7714,7 +7789,7 @@
         <v>153.92403509182</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>168.9</v>
@@ -7729,12 +7804,12 @@
         <v>520.915579880215</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>33222.9</v>
@@ -7779,44 +7854,44 @@
         <v>490.0706</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>33222.9</v>
@@ -7827,28 +7902,28 @@
       <c r="D10" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="7" t="n">
         <v>39.4372585838387</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="7" t="n">
         <v>5.70230308629154</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G10" s="7" t="n">
         <v>2.54228147539589</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H10" s="7" t="n">
         <v>0.464784237905866</v>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="I10" s="7" t="n">
         <v>16.9768730494089</v>
       </c>
-      <c r="J10" s="6" t="n">
+      <c r="J10" s="7" t="n">
         <v>24.9770892950197</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>21495.3</v>
@@ -7859,28 +7934,28 @@
       <c r="D11" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="7" t="n">
         <v>0.556888327919477</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="7" t="n">
         <v>0.373256864797872</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="7" t="n">
         <v>0.195812568197149</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="H11" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="I11" s="7" t="n">
         <v>22.9911075058746</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>33222.9</v>
@@ -7891,28 +7966,28 @@
       <c r="D12" s="2" t="n">
         <v>0.2</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="7" t="n">
         <v>0.908874182659571</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="7" t="n">
         <v>0.514565682603055</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="7" t="n">
         <v>0.283055000975135</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="I12" s="7" t="n">
         <v>23.9667529712611</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>21495.3</v>
@@ -7923,28 +7998,28 @@
       <c r="D13" s="2" t="n">
         <v>0.2</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="7" t="n">
         <v>0.00565241433061335</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>33222.9</v>
@@ -7955,28 +8030,28 @@
       <c r="D14" s="2" t="n">
         <v>0.1</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="7" t="n">
         <v>0.00735722463359847</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>33222.9</v>
@@ -7987,28 +8062,28 @@
       <c r="D15" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="E15" s="7" t="n">
         <v>34.4537315506632</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="7" t="n">
         <v>5.36641142272815</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="7" t="n">
         <v>2.45736267961699</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="7" t="n">
         <v>0.502713407094315</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="7" t="n">
         <v>6.45239521409972</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="J15" s="7" t="n">
         <v>11.6478170961914</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>33222.9</v>
@@ -8019,28 +8094,28 @@
       <c r="D16" s="2" t="n">
         <v>0.2</v>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" s="7" t="n">
         <v>0.887488878554445</v>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F16" s="7" t="n">
         <v>0.50490658607203</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G16" s="7" t="n">
         <v>0.251684565516942</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I16" s="7" t="n">
         <v>10.4706385650631</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>21495.3</v>
@@ -8051,23 +8126,23 @@
       <c r="D17" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="E17" s="6" t="n">
+      <c r="E17" s="7" t="n">
         <v>0.589585671823979</v>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F17" s="7" t="n">
         <v>0.398408667801335</v>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G17" s="7" t="n">
         <v>0.208437662459761</v>
       </c>
-      <c r="H17" s="6" t="n">
+      <c r="H17" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="6" t="n">
+      <c r="I17" s="7" t="n">
         <v>8.84197793287098</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>